<commit_message>
Updated str_tempalte.xlsx and added named_manager.py
</commit_message>
<xml_diff>
--- a/templates/str_template.xlsx
+++ b/templates/str_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joseph.adogeri\Desktop\source\supplemental_tax_rolls_generator\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD9212A-A41E-4AE9-8DF8-C0F0C9D1466A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D986258-2B08-44AA-A7EA-D986BCBAF0DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1245" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20820" yWindow="5265" windowWidth="16875" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONSOLIDATED SUMMARY" sheetId="3" r:id="rId1"/>
@@ -972,24 +972,24 @@
         <v>7</v>
       </c>
       <c r="B14" s="24">
-        <f>SUM(B12,ABS(B13))</f>
+        <f>SUM(B12 - ABS(B13))</f>
+        <v>10000</v>
+      </c>
+      <c r="C14" s="24">
+        <f>SUM(C12 - ABS(C13))</f>
+        <v>20000</v>
+      </c>
+      <c r="D14" s="24">
+        <f>SUM(D12 - ABS(D13))</f>
         <v>30000</v>
       </c>
-      <c r="C14" s="24">
-        <f>SUM(C12,ABS(C13))</f>
-        <v>60000</v>
-      </c>
-      <c r="D14" s="24">
-        <f>SUM(D12,ABS(D13))</f>
-        <v>90000</v>
-      </c>
       <c r="E14" s="24">
-        <f>SUM(E12,ABS(E13))</f>
-        <v>120000</v>
+        <f>SUM(E12 - ABS(E13))</f>
+        <v>40000</v>
       </c>
       <c r="F14" s="25">
         <f>SUM(B14:E14)</f>
-        <v>300000</v>
+        <v>100000</v>
       </c>
       <c r="G14" s="14"/>
     </row>

</xml_diff>